<commit_message>
ECS-79 fix load-test report xls template
</commit_message>
<xml_diff>
--- a/eca-load-tests/src/main/resources/templates/load-test-report-template.xlsx
+++ b/eca-load-tests/src/main/resources/templates/load-test-report-template.xlsx
@@ -1,44 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="204" yWindow="564" windowWidth="30396" windowHeight="13164"/>
+  </bookViews>
   <sheets>
-    <sheet name="Отчет по нагрузочному тестирова" r:id="rId1" sheetId="1" state="visible"/>
-    <sheet name="Лист2" r:id="rId2" sheetId="2" state="visible"/>
-    <sheet name="Лист3" r:id="rId3" sheetId="3" state="visible"/>
+    <sheet name="Отчет по нагрузочному тестирова" sheetId="1" r:id="rId1"/>
+    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
+    <sheet name="Лист3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <calcPr calcId="124519"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author/>
+    <author>Пользователь Windows</author>
   </authors>
   <commentList>
-    <comment authorId="0" ref="A1">
+    <comment ref="A1" authorId="0">
       <text>
         <r>
           <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <b val="true"/>
-            <color rgb="000000" tint="0"/>
-            <sz val="9"/>
+            <charset val="1"/>
           </rPr>
-          <t>Roman93:</t>
-        </r>
-        <r>
-          <t xml:space="preserve">
-</t>
+          <t>Пользователь Windows:</t>
         </r>
         <r>
           <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <color rgb="000000" tint="0"/>
-            <sz val="9"/>
+            <charset val="1"/>
           </rPr>
-          <t>jx:area(lastCell="B15")</t>
+          <t xml:space="preserve">
+jx:area(lastCell="B15")</t>
         </r>
       </text>
     </comment>
@@ -47,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Отчет по нагрузочному тестированию</t>
   </si>
@@ -133,27 +137,37 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
-  <numFmts>
-    <numFmt co:extendedFormatCode="General" formatCode="General" numFmtId="1000"/>
-  </numFmts>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="5">
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <color rgb="000000" tint="0"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <b val="true"/>
-      <color rgb="000000" tint="0"/>
-      <sz val="12"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <b val="true"/>
-      <color rgb="000000" tint="0"/>
-      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -165,76 +179,78 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="B9CDE5" tint="0"/>
+        <fgColor rgb="FFB9CDE5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="DCE6F2" tint="0"/>
+        <fgColor rgb="FFDCE6F2"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="3">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
-      <left style="none"/>
+      <left/>
       <right style="thin">
-        <color rgb="000000" tint="0"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="000000" tint="0"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="000000" tint="0"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="000000" tint="0"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="000000" tint="0"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="000000" tint="0"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="000000" tint="0"/>
+        <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="0" numFmtId="1000" quotePrefix="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="0" numFmtId="1000" quotePrefix="false"/>
-    <xf applyFill="true" applyFont="true" applyNumberFormat="true" borderId="0" fillId="2" fontId="1" numFmtId="1000" quotePrefix="false"/>
-    <xf applyFill="true" applyFont="true" applyNumberFormat="true" borderId="0" fillId="3" fontId="1" numFmtId="1000" quotePrefix="false"/>
-    <xf applyFill="true" applyFont="true" applyNumberFormat="true" borderId="0" fillId="3" fontId="0" numFmtId="1000" quotePrefix="false"/>
-    <xf applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="1" fillId="3" fontId="1" numFmtId="1000" quotePrefix="false"/>
-    <xf applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="2" fillId="3" fontId="2" numFmtId="1000" quotePrefix="false"/>
-    <xf applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="2" fillId="3" fontId="0" numFmtId="1000" quotePrefix="false"/>
-    <xf applyBorder="true" applyFill="true" applyFont="true" applyNumberFormat="true" borderId="2" fillId="3" fontId="1" numFmtId="1000" quotePrefix="false"/>
-    <xf applyAlignment="true" applyFont="true" applyNumberFormat="true" borderId="0" fillId="0" fontId="2" numFmtId="1000" quotePrefix="false">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" name="Normal" xfId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleMedium4" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
   <a:themeElements>
     <a:clrScheme name="Стандартная">
       <a:dk1>
@@ -434,318 +450,184 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
-  <sheetPr>
-    <outlinePr summaryBelow="true" summaryRight="true"/>
-  </sheetPr>
-  <dimension ref="A1:AMD23"/>
-  <sheetFormatPr baseColWidth="8" customHeight="false" defaultColWidth="9.14062530925693" defaultRowHeight="14.3999996185303" zeroHeight="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col customWidth="true" max="1" min="1" outlineLevel="0" width="43.6640623533012"/>
-    <col customWidth="true" max="2" min="2" outlineLevel="0" width="40.2187508193987"/>
-    <col customWidth="true" max="3" min="3" outlineLevel="0" width="26.9999998308338"/>
-    <col customWidth="true" max="4" min="4" outlineLevel="0" width="30.8867187123341"/>
-    <col customWidth="true" max="5" min="5" outlineLevel="0" width="34.3320302462366"/>
-    <col customWidth="true" max="6" min="6" outlineLevel="0" width="31.4414051484374"/>
-    <col customWidth="true" max="7" min="7" outlineLevel="0" width="31.5546869436019"/>
-    <col customWidth="true" max="1018" min="8" outlineLevel="0" width="8.55468778943276"/>
+    <col min="1" max="1" width="43.6640625" customWidth="1"/>
+    <col min="2" max="2" width="40.21875" customWidth="1"/>
+    <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="4" max="4" width="30.88671875" customWidth="1"/>
+    <col min="5" max="5" width="34.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.44140625" customWidth="1"/>
+    <col min="7" max="7" width="31.5546875" customWidth="1"/>
+    <col min="8" max="1018" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row ht="15.6000003814697" outlineLevel="0" r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" ht="15.6">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s"/>
-      <c r="C1" s="0" t="n"/>
-      <c r="D1" s="0" t="n"/>
-      <c r="E1" s="0" t="n"/>
-      <c r="F1" s="0" t="n"/>
-      <c r="G1" s="0" t="n"/>
-    </row>
-    <row ht="15.6000003814697" outlineLevel="0" r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="0" t="n"/>
-      <c r="D2" s="0" t="n"/>
-      <c r="E2" s="0" t="n"/>
-      <c r="F2" s="0" t="n"/>
-      <c r="G2" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="3" s="0">
-      <c r="A3" s="4" t="s">
+      <c r="B1" s="8"/>
+    </row>
+    <row r="2" spans="1:2" ht="15.6">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:2" ht="15.6">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="n"/>
-      <c r="D3" s="0" t="n"/>
-      <c r="E3" s="0" t="n"/>
-      <c r="F3" s="0" t="n"/>
-      <c r="G3" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="4" s="0">
-      <c r="A4" s="4" t="s">
+    </row>
+    <row r="4" spans="1:2" ht="15.6">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="0" t="n"/>
-      <c r="D4" s="0" t="n"/>
-      <c r="E4" s="0" t="n"/>
-      <c r="F4" s="0" t="n"/>
-      <c r="G4" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="5" s="0">
-      <c r="A5" s="4" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="15.6">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="0" t="n"/>
-      <c r="D5" s="0" t="n"/>
-      <c r="E5" s="0" t="n"/>
-      <c r="F5" s="0" t="n"/>
-      <c r="G5" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="6" s="0">
-      <c r="A6" s="4" t="s">
+    </row>
+    <row r="6" spans="1:2" ht="15.6">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="0" t="n"/>
-      <c r="D6" s="0" t="n"/>
-      <c r="E6" s="0" t="n"/>
-      <c r="F6" s="0" t="n"/>
-      <c r="G6" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="7" s="0">
-      <c r="A7" s="4" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="15.6">
+      <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="0" t="n"/>
-      <c r="D7" s="0" t="n"/>
-      <c r="E7" s="0" t="n"/>
-      <c r="F7" s="0" t="n"/>
-      <c r="G7" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="8" s="0">
-      <c r="A8" s="4" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="15.6">
+      <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="0" t="n"/>
-      <c r="D8" s="0" t="n"/>
-      <c r="E8" s="0" t="n"/>
-      <c r="F8" s="0" t="n"/>
-      <c r="G8" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="9" s="0">
-      <c r="A9" s="4" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="15.6">
+      <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="0" t="n"/>
-      <c r="D9" s="0" t="n"/>
-      <c r="E9" s="0" t="n"/>
-      <c r="F9" s="0" t="n"/>
-      <c r="G9" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="10" s="0">
-      <c r="A10" s="4" t="s">
+    </row>
+    <row r="10" spans="1:2" ht="15.6">
+      <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="0" t="n"/>
-      <c r="D10" s="0" t="n"/>
-      <c r="E10" s="0" t="n"/>
-      <c r="F10" s="0" t="n"/>
-      <c r="G10" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="11" s="0">
-      <c r="A11" s="4" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="15.6">
+      <c r="A11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="0" t="n"/>
-      <c r="D11" s="0" t="n"/>
-      <c r="E11" s="0" t="n"/>
-      <c r="F11" s="0" t="n"/>
-      <c r="G11" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="12" s="0">
-      <c r="A12" s="4" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="15.6">
+      <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="0" t="n"/>
-      <c r="D12" s="0" t="n"/>
-      <c r="E12" s="0" t="n"/>
-      <c r="F12" s="0" t="n"/>
-      <c r="G12" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="13" s="0">
-      <c r="A13" s="4" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="15.6">
+      <c r="A13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="0" t="n"/>
-      <c r="D13" s="0" t="n"/>
-      <c r="E13" s="0" t="n"/>
-      <c r="F13" s="0" t="n"/>
-      <c r="G13" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="14" s="0">
-      <c r="A14" s="4" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="15.6">
+      <c r="A14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="0" t="n"/>
-      <c r="D14" s="0" t="n"/>
-      <c r="E14" s="0" t="n"/>
-      <c r="F14" s="0" t="n"/>
-      <c r="G14" s="0" t="n"/>
-    </row>
-    <row customFormat="true" ht="15.6000003814697" outlineLevel="0" r="15" s="0">
-      <c r="A15" s="7" t="s">
+    </row>
+    <row r="15" spans="1:2" ht="15.6">
+      <c r="A15" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="0" t="n"/>
-      <c r="D15" s="0" t="n"/>
-      <c r="E15" s="0" t="n"/>
-      <c r="F15" s="0" t="n"/>
-      <c r="G15" s="0" t="n"/>
-    </row>
-    <row customFormat="true" customHeight="true" ht="14.8500003814697" outlineLevel="0" r="16" s="0">
-      <c r="A16" s="0" t="n"/>
-      <c r="B16" s="0" t="n"/>
-      <c r="C16" s="0" t="n"/>
-      <c r="D16" s="0" t="n"/>
-      <c r="E16" s="0" t="n"/>
-      <c r="F16" s="0" t="n"/>
-      <c r="G16" s="0" t="n"/>
-    </row>
-    <row customFormat="true" customHeight="true" ht="14.8500003814697" outlineLevel="0" r="17" s="0">
-      <c r="A17" s="0" t="n"/>
-      <c r="B17" s="0" t="n"/>
-      <c r="C17" s="0" t="n"/>
-      <c r="D17" s="0" t="n"/>
-      <c r="E17" s="0" t="n"/>
-      <c r="F17" s="0" t="n"/>
-      <c r="G17" s="0" t="n"/>
-    </row>
-    <row customFormat="true" customHeight="true" ht="14.8500003814697" outlineLevel="0" r="18" s="0">
-      <c r="A18" s="0" t="n"/>
-      <c r="B18" s="0" t="n"/>
-      <c r="C18" s="0" t="n"/>
-      <c r="D18" s="0" t="n"/>
-      <c r="E18" s="0" t="n"/>
-      <c r="F18" s="0" t="n"/>
-      <c r="G18" s="0" t="n"/>
-    </row>
-    <row customFormat="true" customHeight="true" ht="14.8500003814697" outlineLevel="0" r="19" s="0">
-      <c r="A19" s="0" t="n"/>
-      <c r="B19" s="0" t="n"/>
-      <c r="C19" s="0" t="n"/>
-      <c r="D19" s="0" t="n"/>
-      <c r="E19" s="0" t="n"/>
-      <c r="F19" s="0" t="n"/>
-      <c r="G19" s="0" t="n"/>
-    </row>
-    <row outlineLevel="0" r="20">
-      <c r="C20" s="0" t="n"/>
-      <c r="D20" s="0" t="n"/>
-      <c r="E20" s="0" t="n"/>
-      <c r="F20" s="0" t="n"/>
-      <c r="G20" s="0" t="n"/>
-    </row>
-    <row outlineLevel="0" r="21">
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
-    </row>
-    <row customHeight="true" ht="15" outlineLevel="0" r="22">
-      <c r="C22" s="0" t="n"/>
-      <c r="D22" s="0" t="n"/>
-      <c r="E22" s="0" t="n"/>
-      <c r="F22" s="0" t="n"/>
-      <c r="G22" s="0" t="n"/>
-    </row>
-    <row outlineLevel="0" r="23">
-      <c r="C23" s="0" t="n"/>
-      <c r="D23" s="0" t="n"/>
-      <c r="E23" s="0" t="n"/>
-      <c r="F23" s="0" t="n"/>
-      <c r="G23" s="0" t="n"/>
-    </row>
+    </row>
+    <row r="16" spans="1:2" ht="14.85" customHeight="1"/>
+    <row r="17" spans="3:7" ht="14.85" customHeight="1"/>
+    <row r="18" spans="3:7" ht="14.85" customHeight="1"/>
+    <row r="19" spans="3:7" ht="14.85" customHeight="1"/>
+    <row r="21" spans="3:7">
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+    </row>
+    <row r="22" spans="3:7" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>
-  <pageMargins bottom="0.75" footer="0.511805534362793" header="0.511805534362793" left="0.700000047683716" right="0.700000047683716" top="0.75"/>
-  <pageSetup fitToHeight="0" fitToWidth="0" orientation="portrait" paperHeight="297mm" paperSize="9" paperWidth="210mm" scale="100"/>
+  <pageMargins left="0.70000004768371604" right="0.70000004768371604" top="0.75" bottom="0.75" header="0.51180553436279297" footer="0.51180553436279297"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
-  <sheetPr>
-    <outlinePr summaryBelow="true" summaryRight="true"/>
-  </sheetPr>
-  <dimension ref="A1:AMK1"/>
-  <sheetFormatPr baseColWidth="8" customHeight="false" defaultColWidth="9.14062530925693" defaultRowHeight="14.3999996185303" zeroHeight="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col customWidth="true" max="1025" min="1" outlineLevel="0" width="8.55468778943276"/>
+    <col min="1" max="1025" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData/>
-  <pageMargins bottom="0.75" footer="0.511805534362793" header="0.511805534362793" left="0.700000047683716" right="0.700000047683716" top="0.75"/>
-  <pageSetup fitToHeight="0" fitToWidth="0" orientation="portrait" paperHeight="297mm" paperSize="9" paperWidth="210mm" scale="100"/>
+  <pageMargins left="0.70000004768371604" right="0.70000004768371604" top="0.75" bottom="0.75" header="0.51180553436279297" footer="0.51180553436279297"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:a15="http://schemas.microsoft.com/office/drawing/2012/main" xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:co="http://ncloudtech.com" xmlns:co-ooxml="http://ncloudtech.com/ooxml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/officeDocument/2006/sharedTypes" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main" xmlns:w10="urn:schemas-microsoft-com:office:word" xmlns:w14="http://schemas.microsoft.com/office/word/2010/wordml" xmlns:w15="http://schemas.microsoft.com/office/word/2012/wordml" xmlns:wp="http://schemas.openxmlformats.org/drawingml/2006/wordprocessingDrawing" xmlns:wpg="http://schemas.microsoft.com/office/word/2010/wordprocessingGroup" xmlns:wps="http://schemas.microsoft.com/office/word/2010/wordprocessingShape" xmlns:x="urn:schemas-microsoft-com:office:excel" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" mc:Ignorable="co co-ooxml w14 x14 w15">
-  <sheetPr>
-    <outlinePr summaryBelow="true" summaryRight="true"/>
-  </sheetPr>
-  <dimension ref="A1:AMK1"/>
-  <sheetFormatPr baseColWidth="8" customHeight="false" defaultColWidth="9.14062530925693" defaultRowHeight="14.3999996185303" zeroHeight="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col customWidth="true" max="1025" min="1" outlineLevel="0" width="8.55468778943276"/>
+    <col min="1" max="1025" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData/>
-  <pageMargins bottom="0.75" footer="0.511805534362793" header="0.511805534362793" left="0.700000047683716" right="0.700000047683716" top="0.75"/>
-  <pageSetup fitToHeight="0" fitToWidth="0" orientation="portrait" paperHeight="297mm" paperSize="9" paperWidth="210mm" scale="100"/>
+  <pageMargins left="0.70000004768371604" right="0.70000004768371604" top="0.75" bottom="0.75" header="0.51180553436279297" footer="0.51180553436279297"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>